<commit_message>
add: evods and sqlcondcutor
</commit_message>
<xml_diff>
--- a/src/paper_list.xlsx
+++ b/src/paper_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yizhang/Desktop/Data Agents Survey/awesome-data-agents/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3B5EACC-DC80-FB47-A5F5-371B799325DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E48A0C-52E7-8B40-8E73-2E0BB8420B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="46080" windowHeight="25420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="513">
   <si>
     <t>Category</t>
   </si>
@@ -2416,12 +2416,6 @@
     <t>AgenticData</t>
   </si>
   <si>
-    <t>AgenticData: An Agentic Data Analytics System for Heterogeneous Data</t>
-  </si>
-  <si>
-    <t>https://arxiv.org/pdf/2508.05002</t>
-  </si>
-  <si>
     <t>Tsinghua University</t>
   </si>
   <si>
@@ -2548,22 +2542,42 @@
     <t>Xata</t>
   </si>
   <si>
-    <t>Julius.ai</t>
-  </si>
-  <si>
-    <t>https://julius.ai/</t>
-  </si>
-  <si>
-    <t>Julis</t>
-  </si>
-  <si>
-    <t>Bayeslab.ai</t>
-  </si>
-  <si>
-    <t>https://bayeslab.ai/</t>
-  </si>
-  <si>
-    <t>Bayeslab</t>
+    <t>SQLConductor</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>SQLConductor: Search-to-Policy Learning for Step-wise Text-to-SQL Orchestration</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/pdf/2606.23537</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>AgenticData: A Multi-Agent based Data Analytics System for Heterogeneous Data</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>EvoDS: Self-Evolving Autonomous Data Science Agent with Skill Learning and Context Management</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>EvoDS</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/pdf/2606.03841</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>KDD</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>HKUST(GZ)</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://arxiv.org/pdf/2508.05002v2</t>
+    <phoneticPr fontId="15" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -3462,7 +3476,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -3784,6 +3798,15 @@
     <xf numFmtId="0" fontId="6" fillId="56" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -6648,7 +6671,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K256"/>
+  <dimension ref="A1:K257"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -7520,8 +7543,8 @@
       </c>
     </row>
     <row r="44" spans="1:8" ht="25.25" customHeight="1">
-      <c r="A44" s="3"/>
-      <c r="B44" s="10"/>
+      <c r="A44" s="84"/>
+      <c r="B44" s="107"/>
       <c r="C44" s="65" t="s">
         <v>342</v>
       </c>
@@ -7540,39 +7563,42 @@
     </row>
     <row r="45" spans="1:8" ht="25.25" customHeight="1">
       <c r="A45" s="3"/>
-      <c r="B45" s="11" t="s">
-        <v>146</v>
-      </c>
-      <c r="C45" s="74" t="s">
-        <v>345</v>
-      </c>
-      <c r="D45" s="38" t="s">
-        <v>346</v>
-      </c>
-      <c r="E45" s="38" t="s">
-        <v>347</v>
-      </c>
-      <c r="F45" s="39" t="s">
-        <v>205</v>
-      </c>
-      <c r="G45" s="11">
-        <v>2024</v>
+      <c r="B45" s="10"/>
+      <c r="C45" s="108" t="s">
+        <v>503</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>504</v>
+      </c>
+      <c r="E45" s="109" t="s">
+        <v>505</v>
+      </c>
+      <c r="F45" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="G45" s="10">
+        <v>2026</v>
+      </c>
+      <c r="H45">
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="25.25" customHeight="1">
       <c r="A46" s="3"/>
-      <c r="B46" s="11"/>
-      <c r="C46" s="75" t="s">
-        <v>348</v>
+      <c r="B46" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="C46" s="74" t="s">
+        <v>345</v>
       </c>
       <c r="D46" s="38" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="E46" s="38" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="F46" s="39" t="s">
-        <v>90</v>
+        <v>205</v>
       </c>
       <c r="G46" s="11">
         <v>2024</v>
@@ -7581,117 +7607,117 @@
     <row r="47" spans="1:8" ht="25.25" customHeight="1">
       <c r="A47" s="3"/>
       <c r="B47" s="11"/>
-      <c r="C47" s="74" t="s">
+      <c r="C47" s="75" t="s">
+        <v>348</v>
+      </c>
+      <c r="D47" s="38" t="s">
+        <v>349</v>
+      </c>
+      <c r="E47" s="38" t="s">
+        <v>350</v>
+      </c>
+      <c r="F47" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="G47" s="11">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="25.25" customHeight="1">
+      <c r="A48" s="3"/>
+      <c r="B48" s="11"/>
+      <c r="C48" s="74" t="s">
         <v>351</v>
       </c>
-      <c r="D47" s="38" t="s">
+      <c r="D48" s="38" t="s">
         <v>352</v>
       </c>
-      <c r="E47" s="38" t="s">
+      <c r="E48" s="38" t="s">
         <v>353</v>
       </c>
-      <c r="F47" s="39" t="s">
+      <c r="F48" s="39" t="s">
         <v>205</v>
-      </c>
-      <c r="G47" s="11">
-        <v>2025</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" ht="25.25" customHeight="1">
-      <c r="A48" s="84"/>
-      <c r="B48" s="95"/>
-      <c r="C48" s="75" t="s">
-        <v>354</v>
-      </c>
-      <c r="D48" s="38" t="s">
-        <v>355</v>
-      </c>
-      <c r="E48" s="38" t="s">
-        <v>356</v>
-      </c>
-      <c r="F48" s="39" t="s">
-        <v>154</v>
       </c>
       <c r="G48" s="11">
         <v>2025</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="25.25" customHeight="1">
-      <c r="A49" s="3"/>
-      <c r="B49" s="11"/>
+      <c r="A49" s="84"/>
+      <c r="B49" s="95"/>
       <c r="C49" s="75" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="D49" s="38" t="s">
-        <v>358</v>
-      </c>
-      <c r="E49" s="96" t="s">
-        <v>359</v>
+        <v>355</v>
+      </c>
+      <c r="E49" s="38" t="s">
+        <v>356</v>
       </c>
       <c r="F49" s="39" t="s">
-        <v>17</v>
+        <v>154</v>
       </c>
       <c r="G49" s="11">
-        <v>2026</v>
-      </c>
-      <c r="H49">
-        <v>1</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="25.25" customHeight="1">
       <c r="A50" s="3"/>
-      <c r="B50" s="16" t="s">
-        <v>163</v>
-      </c>
-      <c r="C50" s="58" t="s">
-        <v>360</v>
-      </c>
-      <c r="D50" s="15" t="s">
-        <v>361</v>
-      </c>
-      <c r="E50" s="15" t="s">
-        <v>362</v>
-      </c>
-      <c r="F50" s="33" t="s">
-        <v>136</v>
-      </c>
-      <c r="G50" s="16">
-        <v>2023</v>
+      <c r="B50" s="11"/>
+      <c r="C50" s="75" t="s">
+        <v>357</v>
+      </c>
+      <c r="D50" s="38" t="s">
+        <v>358</v>
+      </c>
+      <c r="E50" s="96" t="s">
+        <v>359</v>
+      </c>
+      <c r="F50" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="G50" s="11">
+        <v>2026</v>
+      </c>
+      <c r="H50">
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="25.25" customHeight="1">
       <c r="A51" s="3"/>
-      <c r="B51" s="16"/>
+      <c r="B51" s="16" t="s">
+        <v>163</v>
+      </c>
       <c r="C51" s="58" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="D51" s="15" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="E51" s="15" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="F51" s="33" t="s">
-        <v>335</v>
+        <v>136</v>
       </c>
       <c r="G51" s="16">
-        <v>2024</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="25.25" customHeight="1">
       <c r="A52" s="3"/>
       <c r="B52" s="16"/>
-      <c r="C52" s="57" t="s">
-        <v>366</v>
+      <c r="C52" s="58" t="s">
+        <v>363</v>
       </c>
       <c r="D52" s="15" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="E52" s="15" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="F52" s="33" t="s">
-        <v>90</v>
+        <v>335</v>
       </c>
       <c r="G52" s="16">
         <v>2024</v>
@@ -7700,17 +7726,17 @@
     <row r="53" spans="1:8" ht="25.25" customHeight="1">
       <c r="A53" s="3"/>
       <c r="B53" s="16"/>
-      <c r="C53" s="58" t="s">
-        <v>369</v>
+      <c r="C53" s="57" t="s">
+        <v>366</v>
       </c>
       <c r="D53" s="15" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="E53" s="15" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="F53" s="33" t="s">
-        <v>123</v>
+        <v>90</v>
       </c>
       <c r="G53" s="16">
         <v>2024</v>
@@ -7720,16 +7746,16 @@
       <c r="A54" s="3"/>
       <c r="B54" s="16"/>
       <c r="C54" s="58" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="D54" s="15" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="E54" s="15" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="F54" s="33" t="s">
-        <v>90</v>
+        <v>123</v>
       </c>
       <c r="G54" s="16">
         <v>2024</v>
@@ -7739,32 +7765,32 @@
       <c r="A55" s="3"/>
       <c r="B55" s="16"/>
       <c r="C55" s="58" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="D55" s="15" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="E55" s="15" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="F55" s="33" t="s">
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="G55" s="16">
-        <v>2025</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="25.25" customHeight="1">
       <c r="A56" s="3"/>
       <c r="B56" s="16"/>
-      <c r="C56" s="57" t="s">
-        <v>378</v>
+      <c r="C56" s="58" t="s">
+        <v>375</v>
       </c>
       <c r="D56" s="15" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="F56" s="33" t="s">
         <v>25</v>
@@ -7777,18 +7803,18 @@
       <c r="A57" s="3"/>
       <c r="B57" s="16"/>
       <c r="C57" s="57" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="D57" s="15" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="E57" s="15" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="F57" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="G57" s="33">
+        <v>25</v>
+      </c>
+      <c r="G57" s="16">
         <v>2025</v>
       </c>
     </row>
@@ -7796,13 +7822,13 @@
       <c r="A58" s="3"/>
       <c r="B58" s="16"/>
       <c r="C58" s="57" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="D58" s="15" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="E58" s="15" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="F58" s="33" t="s">
         <v>13</v>
@@ -7812,94 +7838,94 @@
       </c>
     </row>
     <row r="59" spans="1:8" ht="25.25" customHeight="1">
-      <c r="A59" s="42"/>
-      <c r="B59" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="C59" s="68" t="s">
-        <v>387</v>
-      </c>
-      <c r="D59" s="18" t="s">
-        <v>388</v>
-      </c>
-      <c r="E59" s="24" t="s">
-        <v>389</v>
-      </c>
-      <c r="F59" s="21" t="s">
-        <v>90</v>
-      </c>
-      <c r="G59" s="43">
-        <v>2024</v>
+      <c r="A59" s="3"/>
+      <c r="B59" s="16"/>
+      <c r="C59" s="57" t="s">
+        <v>384</v>
+      </c>
+      <c r="D59" s="15" t="s">
+        <v>385</v>
+      </c>
+      <c r="E59" s="15" t="s">
+        <v>386</v>
+      </c>
+      <c r="F59" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="G59" s="33">
+        <v>2025</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="25.25" customHeight="1">
       <c r="A60" s="42"/>
-      <c r="B60" s="43"/>
-      <c r="C60" s="76" t="s">
-        <v>390</v>
+      <c r="B60" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C60" s="68" t="s">
+        <v>387</v>
       </c>
       <c r="D60" s="18" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="E60" s="24" t="s">
-        <v>392</v>
-      </c>
-      <c r="F60" s="25" t="s">
-        <v>393</v>
+        <v>389</v>
+      </c>
+      <c r="F60" s="21" t="s">
+        <v>90</v>
       </c>
       <c r="G60" s="43">
         <v>2024</v>
       </c>
     </row>
-    <row r="61" spans="1:8">
+    <row r="61" spans="1:8" ht="25.25" customHeight="1">
       <c r="A61" s="42"/>
       <c r="B61" s="43"/>
       <c r="C61" s="76" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="D61" s="18" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="E61" s="24" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="F61" s="25" t="s">
-        <v>190</v>
+        <v>393</v>
       </c>
       <c r="G61" s="43">
         <v>2024</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="25.25" customHeight="1">
+    <row r="62" spans="1:8">
       <c r="A62" s="42"/>
       <c r="B62" s="43"/>
-      <c r="C62" s="68" t="s">
-        <v>397</v>
+      <c r="C62" s="76" t="s">
+        <v>394</v>
       </c>
       <c r="D62" s="18" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="E62" s="24" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="F62" s="25" t="s">
-        <v>13</v>
+        <v>190</v>
       </c>
       <c r="G62" s="43">
-        <v>2025</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="63" spans="1:8" ht="25.25" customHeight="1">
       <c r="A63" s="42"/>
       <c r="B63" s="43"/>
       <c r="C63" s="68" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="D63" s="18" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="E63" s="24" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="F63" s="25" t="s">
         <v>13</v>
@@ -7908,20 +7934,20 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="64" spans="1:8">
+    <row r="64" spans="1:8" ht="25.25" customHeight="1">
       <c r="A64" s="42"/>
       <c r="B64" s="43"/>
-      <c r="C64" s="76" t="s">
-        <v>403</v>
+      <c r="C64" s="68" t="s">
+        <v>400</v>
       </c>
       <c r="D64" s="18" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="E64" s="24" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="F64" s="25" t="s">
-        <v>190</v>
+        <v>13</v>
       </c>
       <c r="G64" s="43">
         <v>2025</v>
@@ -7931,16 +7957,16 @@
       <c r="A65" s="42"/>
       <c r="B65" s="43"/>
       <c r="C65" s="76" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="D65" s="18" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="E65" s="24" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="F65" s="25" t="s">
-        <v>154</v>
+        <v>190</v>
       </c>
       <c r="G65" s="43">
         <v>2025</v>
@@ -7950,16 +7976,16 @@
       <c r="A66" s="42"/>
       <c r="B66" s="43"/>
       <c r="C66" s="76" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="D66" s="18" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="E66" s="24" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="F66" s="25" t="s">
-        <v>190</v>
+        <v>154</v>
       </c>
       <c r="G66" s="43">
         <v>2025</v>
@@ -7969,38 +7995,48 @@
       <c r="A67" s="42"/>
       <c r="B67" s="43"/>
       <c r="C67" s="76" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="D67" s="18" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="E67" s="24" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="F67" s="25" t="s">
-        <v>154</v>
+        <v>190</v>
       </c>
       <c r="G67" s="43">
         <v>2025</v>
       </c>
     </row>
-    <row r="68" spans="1:7" ht="16">
-      <c r="A68" s="4"/>
-      <c r="B68" s="4"/>
-      <c r="C68" s="72"/>
-      <c r="D68" s="44"/>
-      <c r="E68" s="5"/>
-      <c r="F68" s="37"/>
-      <c r="G68" s="4"/>
-    </row>
-    <row r="69" spans="1:7">
+    <row r="68" spans="1:7">
+      <c r="A68" s="42"/>
+      <c r="B68" s="43"/>
+      <c r="C68" s="76" t="s">
+        <v>412</v>
+      </c>
+      <c r="D68" s="18" t="s">
+        <v>413</v>
+      </c>
+      <c r="E68" s="24" t="s">
+        <v>414</v>
+      </c>
+      <c r="F68" s="25" t="s">
+        <v>154</v>
+      </c>
+      <c r="G68" s="43">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="16">
       <c r="A69" s="4"/>
       <c r="B69" s="4"/>
       <c r="C69" s="72"/>
-      <c r="D69" s="46"/>
-      <c r="E69" s="46"/>
-      <c r="F69" s="45"/>
-      <c r="G69" s="47"/>
+      <c r="D69" s="44"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="37"/>
+      <c r="G69" s="4"/>
     </row>
     <row r="70" spans="1:7">
       <c r="A70" s="4"/>
@@ -8042,10 +8078,10 @@
       <c r="A74" s="4"/>
       <c r="B74" s="4"/>
       <c r="C74" s="72"/>
-      <c r="D74" s="5"/>
-      <c r="E74" s="5"/>
-      <c r="F74" s="37"/>
-      <c r="G74" s="4"/>
+      <c r="D74" s="46"/>
+      <c r="E74" s="46"/>
+      <c r="F74" s="45"/>
+      <c r="G74" s="47"/>
     </row>
     <row r="75" spans="1:7">
       <c r="A75" s="4"/>
@@ -9685,15 +9721,27 @@
       <c r="F256" s="37"/>
       <c r="G256" s="4"/>
     </row>
+    <row r="257" spans="1:7">
+      <c r="A257" s="4"/>
+      <c r="B257" s="4"/>
+      <c r="C257" s="72"/>
+      <c r="D257" s="5"/>
+      <c r="E257" s="5"/>
+      <c r="F257" s="37"/>
+      <c r="G257" s="4"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="15" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="E45" r:id="rId1" xr:uid="{9FD907D0-C38C-7440-90E0-75B8454D2F05}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G203"/>
+  <dimension ref="A1:G202"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14" defaultRowHeight="13"/>
   <cols>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -9762,13 +9810,13 @@
         <v>2026</v>
       </c>
       <c r="B4" s="102" t="s">
+        <v>462</v>
+      </c>
+      <c r="C4" s="103" t="s">
+        <v>463</v>
+      </c>
+      <c r="D4" s="104" t="s">
         <v>464</v>
-      </c>
-      <c r="C4" s="103" t="s">
-        <v>465</v>
-      </c>
-      <c r="D4" s="104" t="s">
-        <v>466</v>
       </c>
       <c r="E4" s="101" t="s">
         <v>335</v>
@@ -9802,42 +9850,42 @@
     </row>
     <row r="6" spans="1:7" ht="25.25" customHeight="1">
       <c r="A6" s="37">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B6" s="77" t="s">
         <v>460</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>461</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>462</v>
+      <c r="C6" s="52" t="s">
+        <v>506</v>
+      </c>
+      <c r="D6" s="105" t="s">
+        <v>512</v>
       </c>
       <c r="E6" s="53" t="s">
         <v>13</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="37">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="25.25" customHeight="1">
+      <c r="A7" s="100">
         <v>2026</v>
       </c>
-      <c r="B7" s="77" t="s">
-        <v>467</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>468</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>469</v>
-      </c>
-      <c r="E7" s="53" t="s">
-        <v>123</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>470</v>
+      <c r="B7" s="102" t="s">
+        <v>508</v>
+      </c>
+      <c r="C7" s="71" t="s">
+        <v>507</v>
+      </c>
+      <c r="D7" s="104" t="s">
+        <v>509</v>
+      </c>
+      <c r="E7" s="101" t="s">
+        <v>510</v>
+      </c>
+      <c r="F7" s="103" t="s">
+        <v>511</v>
       </c>
       <c r="G7">
         <v>1</v>
@@ -9845,219 +9893,212 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="37">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B8" s="77" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>473</v>
-      </c>
-      <c r="E8" s="37" t="s">
-        <v>237</v>
+        <v>467</v>
+      </c>
+      <c r="E8" s="53" t="s">
+        <v>123</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>463</v>
+        <v>468</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="37">
         <v>2025</v>
       </c>
-      <c r="B9" s="78" t="s">
-        <v>474</v>
+      <c r="B9" s="77" t="s">
+        <v>469</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>476</v>
-      </c>
-      <c r="E9" s="53" t="s">
-        <v>477</v>
-      </c>
-      <c r="F9" s="52" t="s">
-        <v>463</v>
+        <v>471</v>
+      </c>
+      <c r="E9" s="37" t="s">
+        <v>237</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>461</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="37">
         <v>2025</v>
       </c>
-      <c r="B10" s="77" t="s">
-        <v>478</v>
+      <c r="B10" s="78" t="s">
+        <v>472</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>480</v>
+        <v>474</v>
       </c>
       <c r="E10" s="53" t="s">
-        <v>25</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>481</v>
+        <v>475</v>
+      </c>
+      <c r="F10" s="52" t="s">
+        <v>461</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="37">
+        <v>2025</v>
+      </c>
+      <c r="B11" s="77" t="s">
+        <v>476</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>478</v>
+      </c>
+      <c r="E11" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="37">
         <v>2024</v>
       </c>
-      <c r="B11" s="77" t="s">
+      <c r="B12" s="77" t="s">
+        <v>480</v>
+      </c>
+      <c r="C12" s="52" t="s">
+        <v>481</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>482</v>
       </c>
-      <c r="C11" s="52" t="s">
+      <c r="E12" s="37" t="s">
         <v>483</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="F12" s="52" t="s">
         <v>484</v>
-      </c>
-      <c r="E11" s="37" t="s">
-        <v>485</v>
-      </c>
-      <c r="F11" s="52" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="25.25" customHeight="1">
-      <c r="A12" s="37"/>
-      <c r="B12" s="77" t="s">
-        <v>487</v>
-      </c>
-      <c r="C12" s="52" t="s">
-        <v>488</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>489</v>
-      </c>
-      <c r="E12" s="37"/>
-      <c r="F12" s="5" t="s">
-        <v>490</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="25.25" customHeight="1">
       <c r="A13" s="37"/>
-      <c r="B13" s="78" t="s">
-        <v>491</v>
+      <c r="B13" s="77" t="s">
+        <v>485</v>
       </c>
       <c r="C13" s="52" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>492</v>
+        <v>487</v>
       </c>
       <c r="E13" s="37"/>
       <c r="F13" s="5" t="s">
-        <v>493</v>
+        <v>488</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="25.25" customHeight="1">
       <c r="A14" s="37"/>
       <c r="B14" s="78" t="s">
-        <v>2</v>
+        <v>489</v>
       </c>
       <c r="C14" s="52" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="E14" s="37"/>
       <c r="F14" s="5" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="25.25" customHeight="1">
       <c r="A15" s="37"/>
-      <c r="B15" s="77" t="s">
-        <v>496</v>
+      <c r="B15" s="78" t="s">
+        <v>2</v>
       </c>
       <c r="C15" s="52" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>497</v>
+        <v>492</v>
       </c>
       <c r="E15" s="37"/>
       <c r="F15" s="5" t="s">
-        <v>498</v>
+        <v>493</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="25.25" customHeight="1">
       <c r="A16" s="37"/>
-      <c r="B16" s="78" t="s">
-        <v>499</v>
+      <c r="B16" s="77" t="s">
+        <v>494</v>
       </c>
       <c r="C16" s="52" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>500</v>
+        <v>495</v>
       </c>
       <c r="E16" s="37"/>
       <c r="F16" s="5" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="25.25" customHeight="1">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="25.25" customHeight="1">
       <c r="A17" s="37"/>
-      <c r="B17" s="37" t="s">
-        <v>502</v>
+      <c r="B17" s="78" t="s">
+        <v>497</v>
       </c>
       <c r="C17" s="52" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="E17" s="37"/>
       <c r="F17" s="5" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="25.25" customHeight="1">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="25.25" customHeight="1">
       <c r="A18" s="37"/>
-      <c r="B18" s="53" t="s">
-        <v>505</v>
+      <c r="B18" s="37" t="s">
+        <v>500</v>
       </c>
       <c r="C18" s="52" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>506</v>
+        <v>501</v>
       </c>
       <c r="E18" s="37"/>
       <c r="F18" s="5" t="s">
-        <v>507</v>
-      </c>
-      <c r="G18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19" s="37"/>
-      <c r="B19" s="37" t="s">
-        <v>508</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>488</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>509</v>
-      </c>
+      <c r="B19" s="37"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
       <c r="E19" s="37"/>
-      <c r="F19" s="5" t="s">
-        <v>510</v>
-      </c>
-      <c r="G19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="F19" s="5"/>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20" s="37"/>
       <c r="B20" s="37"/>
       <c r="C20" s="5"/>
@@ -10065,7 +10106,7 @@
       <c r="E20" s="37"/>
       <c r="F20" s="5"/>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:6">
       <c r="A21" s="37"/>
       <c r="B21" s="37"/>
       <c r="C21" s="5"/>
@@ -10073,7 +10114,7 @@
       <c r="E21" s="37"/>
       <c r="F21" s="5"/>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:6">
       <c r="A22" s="37"/>
       <c r="B22" s="37"/>
       <c r="C22" s="5"/>
@@ -10081,7 +10122,7 @@
       <c r="E22" s="37"/>
       <c r="F22" s="5"/>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:6">
       <c r="A23" s="37"/>
       <c r="B23" s="37"/>
       <c r="C23" s="5"/>
@@ -10089,7 +10130,7 @@
       <c r="E23" s="37"/>
       <c r="F23" s="5"/>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:6">
       <c r="A24" s="37"/>
       <c r="B24" s="37"/>
       <c r="C24" s="5"/>
@@ -10097,7 +10138,7 @@
       <c r="E24" s="37"/>
       <c r="F24" s="5"/>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:6">
       <c r="A25" s="37"/>
       <c r="B25" s="37"/>
       <c r="C25" s="5"/>
@@ -10105,7 +10146,7 @@
       <c r="E25" s="37"/>
       <c r="F25" s="5"/>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:6">
       <c r="A26" s="37"/>
       <c r="B26" s="37"/>
       <c r="C26" s="5"/>
@@ -10113,7 +10154,7 @@
       <c r="E26" s="37"/>
       <c r="F26" s="5"/>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:6">
       <c r="A27" s="37"/>
       <c r="B27" s="37"/>
       <c r="C27" s="5"/>
@@ -10121,7 +10162,7 @@
       <c r="E27" s="37"/>
       <c r="F27" s="5"/>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:6">
       <c r="A28" s="37"/>
       <c r="B28" s="37"/>
       <c r="C28" s="5"/>
@@ -10129,7 +10170,7 @@
       <c r="E28" s="37"/>
       <c r="F28" s="5"/>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:6">
       <c r="A29" s="37"/>
       <c r="B29" s="37"/>
       <c r="C29" s="5"/>
@@ -10137,7 +10178,7 @@
       <c r="E29" s="37"/>
       <c r="F29" s="5"/>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:6">
       <c r="A30" s="37"/>
       <c r="B30" s="37"/>
       <c r="C30" s="5"/>
@@ -10145,7 +10186,7 @@
       <c r="E30" s="37"/>
       <c r="F30" s="5"/>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:6">
       <c r="A31" s="37"/>
       <c r="B31" s="37"/>
       <c r="C31" s="5"/>
@@ -10153,7 +10194,7 @@
       <c r="E31" s="37"/>
       <c r="F31" s="5"/>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:6">
       <c r="A32" s="37"/>
       <c r="B32" s="37"/>
       <c r="C32" s="5"/>
@@ -11520,14 +11561,6 @@
       <c r="D202" s="5"/>
       <c r="E202" s="37"/>
       <c r="F202" s="5"/>
-    </row>
-    <row r="203" spans="1:6">
-      <c r="A203" s="37"/>
-      <c r="B203" s="37"/>
-      <c r="C203" s="5"/>
-      <c r="D203" s="5"/>
-      <c r="E203" s="37"/>
-      <c r="F203" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -11540,6 +11573,10 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D6" r:id="rId1" xr:uid="{E0D9AA3D-ED3E-474C-8BB7-59191513ADE6}"/>
+    <hyperlink ref="D7" r:id="rId2" xr:uid="{D47B4A75-6145-064A-B334-6C22DEE8334B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add: representative data agent benchmarks
</commit_message>
<xml_diff>
--- a/src/paper_list.xlsx
+++ b/src/paper_list.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yizhang/Desktop/Data Agents Survey/awesome-data-agents/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E48A0C-52E7-8B40-8E73-2E0BB8420B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C43D8442-FBD6-BB48-83FF-2A3FA5FAB5D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="46080" windowHeight="25420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="46080" windowHeight="25420" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="L1" sheetId="1" r:id="rId1"/>
     <sheet name="L2" sheetId="2" r:id="rId2"/>
     <sheet name="L3" sheetId="3" r:id="rId3"/>
     <sheet name="survey" sheetId="4" r:id="rId4"/>
+    <sheet name="bench" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="532">
   <si>
     <t>Category</t>
   </si>
@@ -2578,6 +2579,70 @@
   <si>
     <t>https://arxiv.org/pdf/2508.05002v2</t>
     <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>DataSpace: Benchmarking Data Agents for Verifiable Analytics over Heterogeneous Workspaces</t>
+  </si>
+  <si>
+    <t>ArXiv</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://arxiv.org/pdf/2608.03451</t>
+  </si>
+  <si>
+    <t>AgenticDataBench: A Comprehensive Benchmark for Data Agents</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/pdf/2607.01647</t>
+  </si>
+  <si>
+    <t>DABstep: Data Agent Benchmark for Multi-step Reasoning</t>
+  </si>
+  <si>
+    <t>ICML</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://arxiv.org/pdf/2606.15300</t>
+  </si>
+  <si>
+    <t>CoDA-Bench: Can Code Agents Handle Data-Intensive Tasks?</t>
+  </si>
+  <si>
+    <t>FDABench: A Benchmark for Data Agents on Analytical Queries over Heterogeneous Data</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/pdf/2509.02473</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://arxiv.org/pdf/2506.23719</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>DAComp: Benchmarking Data Agents across the Full Data Intelligence Lifecycle</t>
+  </si>
+  <si>
+    <t>ICLR</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://arxiv.org/pdf/2512.04324</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>Can AI Agents Answer Your Data Questions? A Benchmark for Data Agents</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/pdf/2603.20576</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>KramaBench: A Benchmark for AI Systems on Data-to-Insight Pipelines over Data Lakes</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/pdf/2506.06541</t>
   </si>
 </sst>
 </file>
@@ -3476,7 +3541,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -3795,9 +3860,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="56" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3805,6 +3867,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="10" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="56" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -7544,7 +7615,7 @@
     </row>
     <row r="44" spans="1:8" ht="25.25" customHeight="1">
       <c r="A44" s="84"/>
-      <c r="B44" s="107"/>
+      <c r="B44" s="106"/>
       <c r="C44" s="65" t="s">
         <v>342</v>
       </c>
@@ -7564,13 +7635,13 @@
     <row r="45" spans="1:8" ht="25.25" customHeight="1">
       <c r="A45" s="3"/>
       <c r="B45" s="10"/>
-      <c r="C45" s="108" t="s">
+      <c r="C45" s="107" t="s">
         <v>503</v>
       </c>
       <c r="D45" s="9" t="s">
         <v>504</v>
       </c>
-      <c r="E45" s="109" t="s">
+      <c r="E45" s="108" t="s">
         <v>505</v>
       </c>
       <c r="F45" s="36" t="s">
@@ -9751,36 +9822,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="109" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="106" t="s">
+      <c r="B1" s="109" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="106" t="s">
+      <c r="C1" s="109" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="106" t="s">
+      <c r="D1" s="109" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="106" t="s">
+      <c r="E1" s="109" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="106" t="s">
+      <c r="F1" s="109" t="s">
         <v>415</v>
       </c>
-      <c r="G1" s="106" t="s">
+      <c r="G1" s="109" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="25.25" customHeight="1">
-      <c r="A2" s="106"/>
-      <c r="B2" s="106"/>
-      <c r="C2" s="106"/>
-      <c r="D2" s="106"/>
-      <c r="E2" s="106"/>
-      <c r="F2" s="106"/>
-      <c r="G2" s="106"/>
+      <c r="A2" s="109"/>
+      <c r="B2" s="109"/>
+      <c r="C2" s="109"/>
+      <c r="D2" s="109"/>
+      <c r="E2" s="109"/>
+      <c r="F2" s="109"/>
+      <c r="G2" s="109"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="37">
@@ -11820,4 +11891,179 @@
   <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D3E3FEC-DF0F-2541-9F0A-5331A96D743D}">
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
+  <cols>
+    <col min="1" max="1" width="13.3984375" customWidth="1"/>
+    <col min="2" max="2" width="52.19921875" customWidth="1"/>
+    <col min="3" max="3" width="38.19921875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="81" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="81" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="81" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="81" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="81" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="82">
+        <v>2026</v>
+      </c>
+      <c r="B2" s="82" t="s">
+        <v>513</v>
+      </c>
+      <c r="C2" s="83" t="s">
+        <v>515</v>
+      </c>
+      <c r="D2" s="82" t="s">
+        <v>514</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="82">
+        <v>2026</v>
+      </c>
+      <c r="B3" t="s">
+        <v>516</v>
+      </c>
+      <c r="C3" s="83" t="s">
+        <v>517</v>
+      </c>
+      <c r="D3" s="82" t="s">
+        <v>514</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="82">
+        <v>2026</v>
+      </c>
+      <c r="B4" t="s">
+        <v>528</v>
+      </c>
+      <c r="C4" s="104" t="s">
+        <v>529</v>
+      </c>
+      <c r="D4" s="82" t="s">
+        <v>514</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="82">
+        <v>2026</v>
+      </c>
+      <c r="B5" t="s">
+        <v>521</v>
+      </c>
+      <c r="C5" s="110" t="s">
+        <v>520</v>
+      </c>
+      <c r="D5" s="71" t="s">
+        <v>519</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="82">
+        <v>2026</v>
+      </c>
+      <c r="B6" t="s">
+        <v>522</v>
+      </c>
+      <c r="C6" s="110" t="s">
+        <v>523</v>
+      </c>
+      <c r="D6" s="71" t="s">
+        <v>510</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="111">
+        <v>2026</v>
+      </c>
+      <c r="B7" t="s">
+        <v>525</v>
+      </c>
+      <c r="C7" s="110" t="s">
+        <v>527</v>
+      </c>
+      <c r="D7" s="71" t="s">
+        <v>526</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="111">
+        <v>2026</v>
+      </c>
+      <c r="B8" t="s">
+        <v>530</v>
+      </c>
+      <c r="C8" s="110" t="s">
+        <v>531</v>
+      </c>
+      <c r="D8" s="71" t="s">
+        <v>526</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="82">
+        <v>2025</v>
+      </c>
+      <c r="B9" t="s">
+        <v>518</v>
+      </c>
+      <c r="C9" s="110" t="s">
+        <v>524</v>
+      </c>
+      <c r="D9" s="82" t="s">
+        <v>514</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="15" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C6" r:id="rId1" xr:uid="{053DDF06-1361-AD41-B096-0870BBCDDF57}"/>
+    <hyperlink ref="C9" r:id="rId2" xr:uid="{2C147D96-0D84-D44C-AAF6-927707DB6BA4}"/>
+    <hyperlink ref="C7" r:id="rId3" xr:uid="{2B6D77A6-1260-6D4A-B44F-D66489DEA31E}"/>
+    <hyperlink ref="C4" r:id="rId4" xr:uid="{FC423275-9CAB-DE4E-ABBA-C9CF1A4EBFF4}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>